<commit_message>
edition-solen-22h: Édition Solen BI 22 h : consolidation du socle, gras PDF, matrice de compétences (point d'étape 3)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modele-binome/catalogue/M09/echantillon/evenements.xlsx
+++ b/modele-binome/catalogue/M09/echantillon/evenements.xlsx
@@ -498,7 +498,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>EV01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -536,7 +536,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>EV02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -612,52 +612,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>EV01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAT1</t>
+          <t>VIP</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>EV01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAT2</t>
+          <t>CAT1</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>EV01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>VIP</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>80</v>
+          <t>CAT2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>35,000</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>EV02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -665,16 +667,14 @@
           <t>CAT1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>50,000</t>
-        </is>
+      <c r="C5" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>EV02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -682,8 +682,10 @@
           <t>CAT2</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>35</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>